<commit_message>
Ala Skateboards satış noktası: 4 materyal baskıya hazır finalize
Teslim: raporlar/ala-materyaller/ (4 PDF, 3mm bleed, gömülü Bebas+Comfortaa,
soc-mavi register). Üretici script: sablonlar/ala-print-materyaller.py.

- Hang tag (60×90mm) · Shelf talker (A5) · A2 poster · QR kart (90×50mm)
- Poster motto: "DÜŞ, KALK, YENİDEN DENE. / Sen de adım at, hareketi sürdür."
- QR → @ayhanerden_ Instagram (error-correction M, taranabilir)
- Render-and-review (5 Haz dersi): 4 kusur yakalandı+düzeltildi
  (logo gri çerçeve artefaktı, 2× footer overlap, Comfortaa-Bold yanlış etiket)
- Türkçe glyph'ler kusursuz (Ş/İ/ç/ş/ı/ğ/ü), ₺ yerine "TL" metni

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sablonlar/SOC_2026_Pazarlama_Plani.xlsx
+++ b/sablonlar/SOC_2026_Pazarlama_Plani.xlsx
@@ -378,7 +378,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -495,6 +495,12 @@
         <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F7"/>
+        <bgColor rgb="00D6E4F7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="68">
     <border>
@@ -1278,7 +1284,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="292">
+  <cellXfs count="294">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2081,6 +2087,10 @@
     <xf numFmtId="0" fontId="50" fillId="0" borderId="44" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3096,9 +3106,32 @@
       <c r="V9" s="72" t="n"/>
       <c r="W9" s="72" t="n"/>
       <c r="X9" s="86" t="n"/>
-      <c r="Y9" s="72" t="n"/>
-      <c r="Z9" s="72" t="n"/>
+      <c r="Y9" s="292" t="inlineStr">
+        <is>
+          <t>ALA SKATEBOARDS KURULUM</t>
+        </is>
+      </c>
+      <c r="Z9" s="292" t="inlineStr">
+        <is>
+          <t>ALA SKT 1. KONTROL</t>
+        </is>
+      </c>
       <c r="AA9" s="63" t="n"/>
+      <c r="AF9" s="293" t="inlineStr">
+        <is>
+          <t>ALA SKT AYLIK ZİYARET</t>
+        </is>
+      </c>
+      <c r="AJ9" s="293" t="inlineStr">
+        <is>
+          <t>ALA SKT AYLIK ZİYARET</t>
+        </is>
+      </c>
+      <c r="AN9" s="293" t="inlineStr">
+        <is>
+          <t>ALA SKT AYLIK ZİYARET</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="79" customHeight="1">
       <c r="A10" s="245" t="n"/>
@@ -3135,6 +3168,11 @@
       <c r="AB10" s="285" t="inlineStr">
         <is>
           <t>LUXMED TEKLİF HAZIRLIĞI</t>
+        </is>
+      </c>
+      <c r="AC10" s="293" t="inlineStr">
+        <is>
+          <t>ALA SKT × TUNCAY İÇERİK ÇEKİMİ</t>
         </is>
       </c>
       <c r="AJ10" s="285" t="inlineStr">
@@ -5386,9 +5424,9 @@
     <mergeCell ref="P3:S3"/>
     <mergeCell ref="AJ4:AM4"/>
     <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A3:C3"/>
     <mergeCell ref="A27:C27"/>
     <mergeCell ref="B15:B17"/>
+    <mergeCell ref="A3:C3"/>
     <mergeCell ref="AR2:AU2"/>
     <mergeCell ref="A26:C26"/>
     <mergeCell ref="A2:C2"/>
@@ -5400,8 +5438,8 @@
     <mergeCell ref="L2:O2"/>
     <mergeCell ref="P4:S4"/>
     <mergeCell ref="X2:AA2"/>
+    <mergeCell ref="A29:C29"/>
     <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A29:C29"/>
     <mergeCell ref="D25:F25"/>
     <mergeCell ref="AJ2:AM2"/>
     <mergeCell ref="D24:F24"/>

</xml_diff>

<commit_message>
xlsx: SOC Faz 2 Strateji kilometre taşları 2026 planına eklendi
- Satır 18 → SOC WEB SİTESİ — TESLİM ZİNCİRİ (açık mavi, Haz–Ağu 12 haftalık milestone)
- Jun W1-W4: menü mimarisi / placeholder kaldır / hero / ekip+iletişim formu
- Jul W1-W4: ajans sayfası / mağaza düzeni / 1. etki hikâyesi / blog ritmi
- Aug W1-W4: email listesi / SEO içerik / etkinlik funnel / GSC baseline
- Yorum: Temmuz W1 (GSC hücresi) strateji çatışması işaretlendi (Ağustos W4'e taşınmalı)

Drive Google Doc (SOC_Strateji_Faz2_2026) paralel yüklendi.
Açık görev #11: Drive native Sheets hâlâ manuel güncelleme bekliyor.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sablonlar/SOC_2026_Pazarlama_Plani.xlsx
+++ b/sablonlar/SOC_2026_Pazarlama_Plani.xlsx
@@ -378,7 +378,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="22">
+  <fills count="23">
     <fill>
       <patternFill/>
     </fill>
@@ -501,6 +501,11 @@
         <bgColor rgb="00D6E4F7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="009DC3E6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="68">
     <border>
@@ -1284,7 +1289,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="294">
+  <cellXfs count="297">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2091,6 +2096,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="22" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2099,6 +2113,25 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors/>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Fox</author>
+  </authors>
+  <commentList>
+    <comment ref="AB12" authorId="0" shapeId="0">
+      <text>
+        <t>⚠️ STRATEJİ ÇATIŞMASI (7 Haz):
+Bu hücrede GSC/Şema bağlantısı Temmuz W1 olarak planlanmış.
+Ancak SOC Strateji Faz 2 (soc-strateji.md) GSC bağlantısını
+Ağustos W4'e erteler (SOC WEB SİTESİ satırına bak).
+Öneri: Bu hücreyi ŞEMA MARKUP olarak bırak; GSC Ağu W4'e taşı.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3528,6 +3561,11 @@
       </c>
     </row>
     <row r="18" ht="137" customHeight="1">
+      <c r="A18" s="294" t="inlineStr">
+        <is>
+          <t>SOC WEB SİTESİ — TESLİM ZİNCİRİ</t>
+        </is>
+      </c>
       <c r="D18" s="47" t="n"/>
       <c r="E18" s="47" t="n"/>
       <c r="F18" s="47" t="n"/>
@@ -3548,11 +3586,66 @@
       <c r="U18" s="47" t="n"/>
       <c r="V18" s="47" t="n"/>
       <c r="W18" s="47" t="n"/>
-      <c r="X18" s="85" t="n"/>
-      <c r="Y18" s="85" t="n"/>
-      <c r="Z18" s="47" t="n"/>
-      <c r="AA18" s="47" t="n"/>
-      <c r="AB18" s="3" t="n"/>
+      <c r="X18" s="295" t="inlineStr">
+        <is>
+          <t>MENÜ MİMARİSİ + KIRIK SAYFA DÜZELTMESİ</t>
+        </is>
+      </c>
+      <c r="Y18" s="295" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER İSTATİSTİK KALDIR</t>
+        </is>
+      </c>
+      <c r="Z18" s="295" t="inlineStr">
+        <is>
+          <t>HERO GÜNCELLEMESİ + HAKKIMIZDA YAYIN</t>
+        </is>
+      </c>
+      <c r="AA18" s="295" t="inlineStr">
+        <is>
+          <t>EKİP SAYFASI + İLETİŞİM FORMU</t>
+        </is>
+      </c>
+      <c r="AB18" s="296" t="inlineStr">
+        <is>
+          <t>AJANS SAYFASI KUR (B2B MESAJ)</t>
+        </is>
+      </c>
+      <c r="AC18" s="295" t="inlineStr">
+        <is>
+          <t>MAĞAZA DÜZENİ (HER ADIM MİSYON)</t>
+        </is>
+      </c>
+      <c r="AD18" s="295" t="inlineStr">
+        <is>
+          <t>1. ETKİ HİKÂYESİ YAYIN</t>
+        </is>
+      </c>
+      <c r="AE18" s="295" t="inlineStr">
+        <is>
+          <t>BLOG RİTMİ BAŞLAT</t>
+        </is>
+      </c>
+      <c r="AF18" s="295" t="inlineStr">
+        <is>
+          <t>EMAİL LİSTESİ + LEAD MAGNET KUR</t>
+        </is>
+      </c>
+      <c r="AG18" s="295" t="inlineStr">
+        <is>
+          <t>SEO İÇERİK (FARKINDALIK + SEKTÖR)</t>
+        </is>
+      </c>
+      <c r="AH18" s="295" t="inlineStr">
+        <is>
+          <t>ETKİNLİK FUNNEL (KAYIT→KATILIM→İÇERİK)</t>
+        </is>
+      </c>
+      <c r="AI18" s="295" t="inlineStr">
+        <is>
+          <t>GSC/ANALYTİCS BAĞLA → BASELINE ÖLÇ</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="127" customHeight="1" thickBot="1">
       <c r="C19" s="60" t="n"/>
@@ -5478,6 +5571,7 @@
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>